<commit_message>
Regenerated API catalogue, touchpoints and data dictionary workbooks; go/no-go and management register
</commit_message>
<xml_diff>
--- a/docs/package/out/BrokerVerse_Communication_Touchpoints.xlsx
+++ b/docs/package/out/BrokerVerse_Communication_Touchpoints.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'E-mails'!$A$1:$P$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Notifications'!$A$1:$G$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'E-mails'!$A$1:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Notifications'!$A$1:$G$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Documents'!$A$1:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Settings'!$A$1:$B$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Operations &gt; Quotation &gt; Quote detail &gt; Share; Operations &gt; Sales &amp; Marketing &gt; Quotations &gt; Coverage detailed view</t>
+          <t>Operations &gt; Sales &amp; Marketing &gt; Quotations &gt; Quote detail &gt; Share; Operations &gt; Sales &amp; Marketing &gt; Quotations &gt; Coverage detailed view</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -700,10 +700,10 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Operations &gt; Quotation &gt; Quote detail &gt; Share</t>
+          <t>Operations &gt; Sales &amp; Marketing &gt; Quotations &gt; Quote detail &gt; Share</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -778,10 +778,10 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -856,10 +856,10 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -934,10 +934,10 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1012,10 +1012,10 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1085,15 +1085,15 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>None (policy schedule PDF downloaded from Policy detail &gt; Policy schedule)</t>
+          <t>Policy schedule PDF (policy-schedule-&lt;policy number&gt;.pdf) when the quotation has a policy</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1168,10 +1168,10 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail); order enforced by renewals.enforce_notice_order</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail); order enforced by renewals.enforce_notice_order</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Premium payment reminder – Policy {{policyNumber}}</t>
+          <t>Premium payment reminder - Policy {{policyNumber}}</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail); the job can be switched off on Master &gt; Schedules</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail); the job can be switched off on Master &gt; Schedules</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Premium payment reminder – Policy {{policyNumber}} (or the subject typed)</t>
+          <t>Premium payment reminder - Policy {{policyNumber}} (or the subject typed)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail); claims.pla_enabled</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail); claims.pla_enabled</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Commission debit note {{dnNumber}} – {{companyName}}</t>
+          <t>Commission debit note {{dnNumber}} - {{companyName}}</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1651,15 +1651,15 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>None, although the body says "Please find our commission debit note"; the PDF is printed from Debit Notes &gt; Print</t>
+          <t>Commission debit note PDF (debit-note-&lt;DN number&gt;.pdf)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1734,10 +1734,10 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1812,10 +1812,10 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -1972,10 +1972,10 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr"/>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>`notification.email_enabled` on and SMTP configured (applies to every e-mail)</t>
+          <t>notification.email_enabled on and SMTP configured (applies to every e-mail)</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2059,8 +2059,164 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Billing and collection</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Official receipt</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Staff click E-mail receipt on a receipt, or automatically when a receipt is recorded and receipts.email_on_record is on.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Accounts &gt; Receipts &gt; View &gt; E-mail receipt</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>The address typed, else the client e-mail; refused with "The client has no e-mail address; enter one" when there is none</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>official-receipt (official-receipt-auto when sent automatically)</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>receipts.email_subject, receipts.email_template, receipts.email_on_record</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Master &gt; Configuration &gt; Billing, Collections &amp; Credit &gt; Receipts</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Official receipt {{receiptNumber}} for policy {{policyNumber}}</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Thank you for your payment. Attached is official receipt &lt;b&gt;{{receiptNumber}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt;.&lt;/p&gt;&lt;table cellpadding="4" style="border-collapse:collapse"&gt;&lt;tr&gt;&lt;td&gt;Amount received&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{amount}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Date received&lt;/td&gt;&lt;td&gt;{{receiptDate}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Mode of payment&lt;/td&gt;&lt;td&gt;{{paymentMode}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Reference&lt;/td&gt;&lt;td&gt;{{referenceNo}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Balance remaining&lt;/td&gt;&lt;td&gt;{{balance}}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;p&gt;{{note}}&lt;/p&gt;&lt;p&gt;Please keep this receipt for your records. If you have any questions about your account, please contact your account officer.&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>clientName, receiptNumber, policyNumber, amount, receiptDate, paymentMode, referenceNo, balance, customerCode, note, companyName</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Official receipt PDF (receipt-&lt;OR number&gt;.pdf)</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>receipts.email_on_record (false) for the automatic e-mail; notification.email_enabled on and SMTP configured</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Billing and collection</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Premium invoice / statement of account</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Staff click E-mail invoice on a collection item, or automatically when a bill is issued from a policy, endorsement or renewal and billing.email_on_issue is on.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Accounts &gt; Collections &gt; Detail &gt; E-mail invoice</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>The address typed, else the client e-mail</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>premium-invoice (premium-invoice-auto when sent automatically)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>billing.email_subject, billing.email_template, billing.payment_instructions, billing.email_on_issue</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Master &gt; Configuration &gt; Other settings &gt; Billing</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Premium invoice {{billNumber}} for policy {{policyNumber}}</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Attached is the premium invoice / statement of account &lt;b&gt;{{billNumber}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; ({{productName}}, {{insurerName}}).&lt;/p&gt;&lt;table cellpadding="4" style="border-collapse:collapse"&gt;&lt;tr&gt;&lt;td&gt;Net premium&lt;/td&gt;&lt;td&gt;{{netPremium}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Taxes and charges&lt;/td&gt;&lt;td&gt;{{taxes}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Gross premium (with taxes)&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{grossPremium}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Amount due&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{amountDue}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Due date&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{dueDate}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;p&gt;{{paymentInstructions}}&lt;/p&gt;&lt;p&gt;{{note}}&lt;/p&gt;&lt;p&gt;Please disregard this notice if payment has already been made. If you have any questions, please contact your account officer.&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>clientName, billNumber, policyNumber, productName, insurerName, netPremium, taxes, grossPremium, amountDue, billDate, dueDate, paymentInstructions, note, companyName</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Premium invoice PDF (invoice-&lt;bill number&gt;.pdf)</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>billing.email_on_issue (false) for the automatic e-mail; notification.email_enabled on and SMTP configured</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P20"/>
+  <autoFilter ref="A1:P22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2071,7 +2227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2207,7 +2363,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Quotation owner</t>
+          <t>Quotation owner (not when they approved it)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2217,17 +2373,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Quotation approved</t>
+          <t>Quotation &lt;number&gt; approved</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Quotation &lt;number&gt; was approved and can be converted to a policy</t>
+          <t>Quotation &lt;number&gt; was approved by &lt;user&gt; and can be converted to a policy</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2474,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Accounting role users</t>
+          <t>Accounting role users except the user who recorded it</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2333,12 +2489,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>&lt;mode&gt; &lt;amount&gt; (ref &lt;reference&gt;) on policy &lt;number&gt;</t>
+          <t>&lt;user&gt; recorded &lt;mode&gt; &lt;amount&gt; (ref &lt;reference&gt;) on policy &lt;number&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2350,32 +2506,32 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Online payment received, failed to apply or amount differs</t>
+          <t>Captured payment confirmed or rejected</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Link creator and roles in payments.notify_roles_on_error (Accounting)</t>
+          <t>User who recorded it</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>task</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Online payment received / Online payment not applied / Online payment to review</t>
+          <t>Premium payment &lt;reference&gt; confirmed / rejected</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;link number&gt;: ... (amount, target and reason)</t>
+          <t>Confirmed by &lt;user&gt; on policy &lt;number&gt;, receipt &lt;OR&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2387,27 +2543,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Collection reminder sent</t>
+          <t>Online payment received, failed to apply or amount differs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Policy owner and holders of write:collections</t>
+          <t>Link creator and roles in payments.notify_roles_on_error (Accounting)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>reminder</t>
+          <t>task</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Premium due &lt;date&gt; – &lt;policy&gt; / Premium overdue &lt;n&gt; day(s) – &lt;policy&gt;</t>
+          <t>Online payment received / Online payment not applied / Online payment to review</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>&lt;client&gt;: &lt;amount&gt; outstanding on &lt;bill&gt;</t>
+          <t>&lt;link number&gt;: ... (amount, target and reason)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2424,27 +2580,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Policy issued over the client credit limit</t>
+          <t>Collection reminder sent</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:collections</t>
+          <t>Policy owner and holders of write:collections</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>reminder</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Client credit limit exceeded</t>
+          <t>Premium due &lt;date&gt; - &lt;policy&gt; / Premium overdue &lt;n&gt; day(s) - &lt;policy&gt;</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;client&gt;: open premium &lt;exposure&gt; is over the credit limit &lt;limit&gt; by &lt;excess&gt; after &lt;policy&gt;</t>
+          <t>&lt;client&gt;: &lt;amount&gt; outstanding on &lt;bill&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2461,27 +2617,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Premium warranty extension requested</t>
+          <t>Policy issued over the client credit limit</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Holders of approve:credit-control</t>
+          <t>Holders of write:collections</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Premium warranty extension to approve</t>
+          <t>Client credit limit exceeded</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;policy&gt; (&lt;client&gt;) until &lt;date&gt;</t>
+          <t>&lt;client&gt;: open premium &lt;exposure&gt; is over the credit limit &lt;limit&gt; by &lt;excess&gt; after &lt;policy&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2498,32 +2654,32 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Premium warranty extension decided</t>
+          <t>Premium warranty extension requested</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Requester</t>
+          <t>Holders of approve:credit-control</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Warranty extension approved / rejected</t>
+          <t>Warranty extension &lt;policy&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;policy&gt; until &lt;date&gt;: &lt;remarks&gt;</t>
+          <t>&lt;user&gt; submitted &lt;policy&gt; (&lt;client&gt;, deadline &lt;date&gt; to &lt;date&gt;: &lt;reason&gt;)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2535,64 +2691,64 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Cancellation for non-payment requested</t>
+          <t>Premium warranty extension decided</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:endorsements</t>
+          <t>Requester</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Cancellation for non-payment requested</t>
+          <t>Warranty extension &lt;policy&gt; approved / rejected</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;policy&gt; (&lt;client&gt;): &lt;endorsement number&gt;</t>
+          <t>Deadline moved to &lt;date&gt;; approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;remarks&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Policy servicing</t>
+          <t>Billing and collection</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Endorsement completed</t>
+          <t>Cancellation for non-payment requested</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Policy owner</t>
+          <t>Holders of write:endorsements</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>action</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Endorsement completed / Policy cancelled by endorsement</t>
+          <t>Cancellation for non-payment requested</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Endorsement &lt;number&gt; on policy &lt;number&gt; was completed (premium change &lt;amount&gt;)</t>
+          <t>&lt;policy&gt; (&lt;client&gt;): &lt;endorsement number&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2604,37 +2760,37 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>Policy servicing</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Claim registered</t>
+          <t>Endorsement completed</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Claim handler and policy owner</t>
+          <t>Policy owner</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>task</t>
+          <t>info</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>New claim &lt;number&gt;</t>
+          <t>Endorsement completed / Policy cancelled by endorsement</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Claim &lt;number&gt; registered on policy &lt;number&gt;</t>
+          <t>Endorsement &lt;number&gt; on policy &lt;number&gt; was completed (premium change &lt;amount&gt;)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>notification.claim_status</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2802,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Claim status changes</t>
+          <t>Claim registered</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2656,17 +2812,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>task</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Claim &lt;number&gt;: &lt;status&gt;</t>
+          <t>New claim &lt;number&gt;</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;note&gt; or "Claim &lt;number&gt; is now &lt;status&gt;"</t>
+          <t>Claim &lt;number&gt; registered on policy &lt;number&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2683,106 +2839,106 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Settlement submitted (maker-checker)</t>
+          <t>Claim status changes</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Claims role users except the submitter</t>
+          <t>Claim handler and policy owner</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>info</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Settlement approval: &lt;claim&gt;</t>
+          <t>Claim &lt;number&gt;: &lt;status&gt;</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Settlement of &lt;amount&gt; on claim &lt;claim&gt; awaits approval</t>
+          <t>&lt;note&gt; or "Claim &lt;number&gt; is now &lt;status&gt;"</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>claims.settlement_maker_checker</t>
+          <t>notification.claim_status</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Renewal notice sent</t>
+          <t>Settlement submitted (maker-checker)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Policy owner</t>
+          <t>Claims role users except the submitter</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>reminder</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>&lt;notice label&gt;: &lt;policy&gt;</t>
+          <t>Claim settlement &lt;claim&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;notice label&gt; sent for policy &lt;policy&gt; expiring &lt;date&gt;</t>
+          <t>&lt;user&gt; submitted &lt;claim&gt; (&lt;amount&gt;, &lt;settlement type&gt;)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>claims.settlement_maker_checker, notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Renewal notices job (60, 30, 15 days)</t>
+          <t>Settlement approved or returned</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Policy owner</t>
+          <t>Submitter</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>reminder</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Renewal due in &lt;n&gt; days</t>
+          <t>Claim settlement &lt;claim&gt; approved / returned</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Policy &lt;number&gt; expires on &lt;date&gt;</t>
+          <t>Approved by &lt;user&gt; / Returned by &lt;user&gt;: &lt;note&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>notification.renewal_reminder</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2794,27 +2950,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Renewal terms submitted</t>
+          <t>Renewal notice sent</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Users with roles in renewals.approver_roles (Processing Team)</t>
+          <t>Policy owner</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>reminder</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Renewal approval: &lt;policy&gt;</t>
+          <t>&lt;notice label&gt;: &lt;policy&gt;</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Renewal &lt;number&gt; (&lt;premium&gt;) awaits approval</t>
+          <t>&lt;notice label&gt; sent for policy &lt;policy&gt; expiring &lt;date&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2831,32 +2987,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Renewal approved or returned</t>
+          <t>Renewal notices job (60, 30, 15 days)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Submitter</t>
+          <t>Policy owner</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>reminder</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Renewal approved / returned: &lt;policy&gt;</t>
+          <t>Renewal due in &lt;n&gt; days</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;note&gt; or "Renewal &lt;number&gt; was approved / returned"</t>
+          <t>Policy &lt;number&gt; expires on &lt;date&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.renewal_reminder</t>
         </is>
       </c>
     </row>
@@ -2868,32 +3024,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Renewal completed</t>
+          <t>Renewal terms submitted</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Policy owner</t>
+          <t>Users with roles in renewals.approver_roles (Processing Team) except the submitter</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Policy renewed: &lt;policy&gt;</t>
+          <t>Renewal &lt;number&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>New term &lt;new policy&gt; from &lt;inception&gt; to &lt;expiry&gt;</t>
+          <t>&lt;user&gt; submitted &lt;number&gt; (policy &lt;policy&gt;, &lt;premium&gt;)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -2905,64 +3061,64 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Renewal lapsed (manual or pipeline job)</t>
+          <t>Renewal approved or returned</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Policy owner</t>
+          <t>Submitter (else the policy owner)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Policy lapsed: &lt;policy&gt;</t>
+          <t>Renewal &lt;number&gt; approved / returned</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;reason&gt;</t>
+          <t>Approved / Returned by &lt;user&gt;: &lt;note&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Remittance and commission</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Remittances submitted for approval</t>
+          <t>Renewal completed</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:remittance</t>
+          <t>Policy owner</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>info</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Remittances awaiting approval</t>
+          <t>Policy renewed: &lt;policy&gt;</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;n&gt; remittance(s) in batch &lt;batch&gt; need approval</t>
+          <t>New term &lt;new policy&gt; from &lt;inception&gt; to &lt;expiry&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2974,32 +3130,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Remittance and commission</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Remittance, settlement or transfer approved or rejected</t>
+          <t>Renewal lapsed (manual or pipeline job)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Initiator</t>
+          <t>Policy owner</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>alert</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>&lt;transaction type&gt; approved / rejected</t>
+          <t>Policy lapsed: &lt;policy&gt;</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>&lt;reference&gt; was approved / rejected by &lt;user&gt;</t>
+          <t>&lt;reason&gt;</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3016,7 +3172,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Commission debit note submitted</t>
+          <t>Remittances submitted for approval</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3031,17 +3187,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Commission debit note awaiting approval</t>
+          <t>Remittance batch &lt;batch&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;DN number&gt; to &lt;insurer&gt; for &lt;amount&gt; needs approval</t>
+          <t>&lt;user&gt; submitted &lt;n&gt; remittance(s) in batch &lt;batch&gt; (&lt;total&gt;)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -3053,32 +3209,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Commission debit note decided</t>
+          <t>Settlement submitted, adjustment needing approval, electronic transfer</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>Holders of write:remittance</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Debit note approved / rejected</t>
+          <t>Settlement / Adjustment / Electronic transfer &lt;reference&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;DN number&gt; to &lt;insurer&gt; was approved / rejected: &lt;reason&gt;</t>
+          <t>&lt;user&gt; submitted &lt;reference&gt; (&lt;description&gt;, &lt;amount&gt;)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -3090,32 +3246,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Incentive calculation submitted</t>
+          <t>Remittance, settlement, adjustment or transfer approved or rejected</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:incentive</t>
+          <t>Initiator</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Incentive calculation awaiting approval</t>
+          <t>&lt;transaction type&gt; &lt;reference&gt; approved / rejected</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;batch&gt; (&lt;period&gt;) needs approval</t>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -3127,234 +3283,234 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Incentive batch decided</t>
+          <t>Commission debit note submitted</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Submitter</t>
+          <t>Holders of write:remittance</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Incentive batch approved / rejected</t>
+          <t>Commission debit note &lt;DN number&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;batch&gt; (&lt;period&gt;)</t>
+          <t>&lt;user&gt; submitted &lt;DN number&gt; (&lt;insurer&gt;, &lt;amount&gt;)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Reinsurance</t>
+          <t>Remittance and commission</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Treaty submitted for approval</t>
+          <t>Commission debit note decided</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:reinsurance</t>
+          <t>Creator</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Treaty awaiting approval</t>
+          <t>Commission debit note &lt;DN number&gt; approved / rejected</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;number&gt; &lt;name&gt; needs approval</t>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Reinsurance</t>
+          <t>Remittance and commission</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Treaty decided</t>
+          <t>Incentive calculation submitted</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Submitter</t>
+          <t>Holders of write:incentive</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Treaty approved / rejected</t>
+          <t>Incentive calculation &lt;batch&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;number&gt; &lt;name&gt;</t>
+          <t>&lt;user&gt; submitted &lt;batch&gt; (period &lt;period&gt;)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Finance and period end</t>
+          <t>Remittance and commission</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher submitted for approval</t>
+          <t>Incentive batch decided</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:journal-vouchers</t>
+          <t>Submitter</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher &lt;number&gt; awaiting approval</t>
+          <t>Incentive calculation &lt;batch&gt; approved / rejected</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;amount&gt;)</t>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Finance and period end</t>
+          <t>Remittance and commission</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher approved</t>
+          <t>Commission lines eligible (marked by a user, or premium fully collected)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>Holders of write:commission</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher &lt;number&gt; approved</t>
+          <t>Commission payout &lt;referrer&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Approved and posted by &lt;user&gt;</t>
+          <t>&lt;user&gt; marked lines eligible / Premium of &lt;policy&gt; fully collected: &lt;n&gt; line(s) of &lt;referrer&gt; awaiting approval (&lt;amount&gt;)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Finance and period end</t>
+          <t>Remittance and commission</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher rejected</t>
+          <t>Commission lines approved</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>User who marked them eligible</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>info</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Journal voucher &lt;number&gt; rejected</t>
+          <t>Commission payout &lt;referrer&gt; approved</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;reason&gt;</t>
+          <t>Approved by &lt;user&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Finance and period end</t>
+          <t>Reinsurance</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Petty cash request submitted</t>
+          <t>Treaty created or changed (reinsurance.treaty_requires_approval)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Holders of write:disbursements</t>
+          <t>Holders of write:reinsurance</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3364,54 +3520,54 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Petty cash request &lt;number&gt; awaiting approval</t>
+          <t>Treaty &lt;number&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>&lt;requester&gt;: &lt;amount&gt;</t>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;name&gt;)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Finance and period end</t>
+          <t>Reinsurance</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Petty cash request decided</t>
+          <t>Treaty decided</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>Submitter</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>info / alert</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Petty cash request &lt;number&gt; approved / rejected</t>
+          <t>Treaty &lt;number&gt; approved / rejected</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;reason&gt; or "By &lt;user&gt;"</t>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -3423,32 +3579,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Petty cash fund below minimum</t>
+          <t>Journal voucher submitted for approval (manual, reversal, correction)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Custodian, holders of write:disbursements</t>
+          <t>Holders of write:journal-vouchers</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Petty cash &lt;code&gt; below minimum</t>
+          <t>Journal voucher &lt;number&gt; awaiting approval</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Available &lt;amount&gt;; minimum cashbox &lt;amount&gt;. Replenish the fund.</t>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;amount&gt;)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
     </row>
@@ -3460,37 +3616,814 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>Bank adjustment journal awaiting approval; year-end adjustment journal (period 13)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Holders of write:journal-vouchers</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Journal voucher &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (bank adjustment: &lt;type&gt;, &lt;amount&gt; / year-end adjustment, period &lt;period&gt;)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Journal voucher approved (Journal Voucher, accounting queue, bank adjustment)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Journal voucher &lt;number&gt; approved</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Approved and posted by &lt;user&gt;</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Journal voucher rejected</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Journal voucher &lt;number&gt; rejected</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Payment voucher submitted for approval (status For approval, agent payout vouchers)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Holders of write:disbursements</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Payment voucher &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;payee&gt;, &lt;amount&gt;)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Payment voucher approved (cheque approved, agent payout approved), or sent back to draft / cancelled while awaiting approval</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Payment voucher &lt;number&gt; approved / rejected / cancelled</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Cheque issued (Pending)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Holders of write:disbursements</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Cheque &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;payee&gt;, &lt;amount&gt;)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Cheque approved or cancelled while Pending</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Cheque &lt;number&gt; approved / cancelled</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Approved / Cancelled by &lt;user&gt;</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash request submitted</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Holders of write:disbursements</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash request &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;requester&gt;, &lt;amount&gt;)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash request decided</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash request &lt;number&gt; approved / rejected</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Posting rule or account determination change requested (accounting.configuration_maker_checker)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Holders of approve:posting-rules</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Configuration change &lt;id&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; requested &lt;kind&gt;: &lt;target&gt; (&lt;note&gt;)</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Configuration change decided</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Requester</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Configuration change &lt;id&gt; approved / rejected</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>&lt;kind&gt;: &lt;target&gt; approved by &lt;user&gt; and in effect / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Insurer reconciliation submitted</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Holders of approve:insurer-reconciliation</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Insurer reconciliation &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;insurer&gt;, &lt;period&gt;, paid &lt;amount&gt;)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Insurer reconciliation decided</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Submitter</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Insurer reconciliation &lt;number&gt; approved / rejected</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Bank reconciliation prepared</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Holders of approve:bank-reconciliation</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Bank reconciliation &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt; (&lt;bank account&gt;, period &lt;period&gt;, bank balance &lt;amount&gt;)</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Bank reconciliation approved, or reopened (rejected when it was prepared)</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Preparer</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Bank reconciliation &lt;number&gt; approved / rejected / reopened</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;remarks&gt;</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Month-end close submitted (accounting.period_close_requires_approval)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Holders of approve:period-end</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Month-end close &lt;number&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; submitted &lt;number&gt;: close / soft close of period &lt;period&gt;</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Month-end close approved or rejected</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Submitter</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Month-end close &lt;number&gt; approved / rejected</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Period &lt;period&gt; closed; approved by &lt;user&gt; / Rejected by &lt;user&gt;: &lt;reason&gt;</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash fund below minimum</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Custodian, holders of write:disbursements</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Petty cash &lt;code&gt; below minimum</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Available &lt;amount&gt;; minimum cashbox &lt;amount&gt;. Replenish the fund.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Finance and period end</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
           <t>Month-end reminder job</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Holders of write:period-end (high priority)</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>reminder</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Month-end close: &lt;period&gt; ends in &lt;n&gt; day(s) / Month-end close: &lt;period&gt; is still open</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Accounting period &lt;period&gt; ends on &lt;date&gt;. Post pending journals and prepare the month-end close run. / ... ended on &lt;date&gt; and is not closed yet.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Job month-end-reminder (off by default)</t>
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Access control</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Authority limit proposed</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Holders of approve:access-control</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Authority limit #&lt;id&gt; awaiting approval</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; proposed &lt;transaction type&gt; for &lt;role or user&gt;: &lt;limit&gt; (&lt;remarks&gt;)</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Access control</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Authority limit decided</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Proposer</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>info / alert</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Authority limit #&lt;id&gt; approved / rejected</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>&lt;transaction type&gt; for &lt;role or user&gt;: &lt;limit&gt;, approved by &lt;user&gt; and in effect / Rejected by &lt;user&gt;: &lt;note&gt;</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Access control</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Access review started</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Holders of write:access-control</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>approval</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Access review &lt;name&gt; awaiting decisions</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>&lt;user&gt; started &lt;name&gt;: &lt;n&gt; user(s) to keep or revoke by &lt;due date&gt;</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>notification.approval_requests</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G38"/>
+  <autoFilter ref="A1:G59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3546,7 +4479,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Operations &gt; Quotation &gt; Quote detail &gt; Share &gt; Download</t>
+          <t>Operations &gt; Sales &amp; Marketing &gt; Quotations &gt; Quote detail &gt; Share &gt; Download</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -3955,7 +4888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3970,506 +4903,506 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value (test system)</t>
+          <t>Value (OOTB seed)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>claims.documents</t>
+          <t>accounting.configuration_maker_checker</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>{"Claims Data Sheet": ["Claim number: {{claimNumber}}", "Policy number: {{policyNumber}}", "Insured: {{insuredName}}", "Insurer: {{insurerName}}", "Line of business: {{lob}}", "Status: {{status}}", "Date of loss: {{lossDate}} {{lossTime}}", "Place of loss: {{lossPlace}}", "Nature of loss: {{lossType}}", "Estimated amount: {{currency}} {{estimate}}", "Approved amount: {{currency}} {{approvedAmount}}", "Settled amount: {{currency}} {{settledAmount}}"], "Claims Discharge Voucher": ["Claim {{claimNumber}} under policy {{policyNumber}}", "Insured: {{insuredName}}", "Settlement amount: {{currency}} {{settledAmount}}", "Settlement type: {{settlementType}}", "I accept the above amount in full and final settlement of this claim.", "Signature: ______________________   Date: ____________"], "Claims Acknowledgement Letter": ["We acknowledge receipt of your claim {{claimNumber}} under policy {{policyNumber}}.", "Insured: {{insuredName}}", "Date of loss: {{lossDate}}", "Reported on: {{reportedDate}}", "Our claims team will contact you within {{slaDays}} days."]}</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>claims.pla_default_recipient</t>
+          <t>accounting.period_close_requires_approval</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>"claims@brokerverse.local"</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>claims.pla_enabled</t>
+          <t>billing.email_on_issue</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>claims.pla_subject</t>
+          <t>billing.email_subject</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>"Preliminary Loss Advice - {{claimNumber}} / {{policyNumber}}"</t>
+          <t>"Premium invoice {{billNumber}} for policy {{policyNumber}}"</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>claims.pla_template</t>
+          <t>billing.email_template</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Dear {{insurerName}},&lt;/p&gt;&lt;p&gt;We advise a loss under policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; of {{insuredName}}.&lt;/p&gt;&lt;p&gt;Claim reference: {{claimNumber}}&lt;br/&gt;Date of loss: {{lossDate}} {{lossTime}}&lt;br/&gt;Place of loss: {{lossPlace}}&lt;br/&gt;Nature of loss: {{lossType}}&lt;br/&gt;Estimated amount: {{currency}} {{estimate}}&lt;/p&gt;&lt;p&gt;{{message}}&lt;/p&gt;&lt;p&gt;{{companyName}} Claims&lt;/p&gt;"</t>
+          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Attached is the premium invoice / statement of account &lt;b&gt;{{billNumber}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; ({{productName}}, {{insurerName}}).&lt;/p&gt;&lt;table cellpadding=\"4\" style=\"border-collapse:collapse\"&gt;&lt;tr&gt;&lt;td&gt;Net premium&lt;/td&gt;&lt;td&gt;{{netPremium}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Taxes and charges&lt;/td&gt;&lt;td&gt;{{taxes}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Gross premium (with taxes)&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{grossPremium}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Amount due&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{amountDue}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Due date&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{dueDate}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;p&gt;{{paymentInstructions}}&lt;/p&gt;&lt;p&gt;{{note}}&lt;/p&gt;&lt;p&gt;Please disregard this notice if payment has already been made. If you have any questions, please contact your account officer.&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;"</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>collections.email_subject</t>
+          <t>billing.payment_instructions</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>"Premium payment reminder – Policy {{policyNumber}}"</t>
+          <t>"Please settle the amount due on or before the due date. Make cheques payable to {{companyName}} and quote bill number {{billNumber}} as the payment reference. For bank transfers or e-wallet payments, please send the proof of payment to your account officer."</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>collections.email_template</t>
+          <t>claims.documents</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;This is a friendly reminder that the premium of &lt;b&gt;{{amount}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; (bill {{billNumber}}) is due on {{dueDate}}.&lt;/p&gt;&lt;p&gt;Please disregard this notice if payment has been made.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+          <t>{"Claims Data Sheet": ["Claim number: {{claimNumber}}", "Policy number: {{policyNumber}}", "Insured: {{insuredName}}", "Insurer: {{insurerName}}", "Line of business: {{lob}}", "Status: {{status}}", "Date of loss: {{lossDate}} {{lossTime}}", "Place of loss: {{lossPlace}}", "Nature of loss: {{lossType}}", "Estimated amount: {{currency}} {{estimate}}", "Approved amount: {{currency}} {{approvedAmount}}", "Settled amount: {{currency}} {{settledAmount}}"], "Claims Discharge Voucher": ["Claim {{claimNumber}} under policy {{policyNumber}}", "Insured: {{insuredName}}", "Settlement amount: {{currency}} {{settledAmount}}", "Settlement type: {{settlementType}}", "I accept the above amount in full and final settlement of this claim.", "Signature: ______________________   Date: ____________"], "Claims Acknowledgement Letter": ["We acknowledge receipt of your claim {{claimNumber}} under policy {{policyNumber}}.", "Insured: {{insuredName}}", "Date of loss: {{lossDate}}", "Reported on: {{reportedDate}}", "Our claims team will contact you within {{slaDays}} days."]}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>collections.reminder_days_before</t>
+          <t>claims.pla_default_recipient</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>"claims@brokerverse.local"</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>collections.reminder_repeat_days</t>
+          <t>claims.pla_enabled</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>direct_bill.email_body</t>
+          <t>claims.pla_subject</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Dear {{insurerName}},&lt;/p&gt;&lt;p&gt;Please find our commission debit note &lt;b&gt;{{dnNumber}}&lt;/b&gt; for {{amount}}, due on {{dueDate}}.&lt;/p&gt;&lt;p&gt;Kindly settle the amount net of the expanded withholding tax on the commission and send BIR Form 2307 for the tax withheld.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+          <t>"Preliminary Loss Advice - {{claimNumber}} / {{policyNumber}}"</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>direct_bill.email_subject</t>
+          <t>claims.pla_template</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>"Commission debit note {{dnNumber}} – {{companyName}}"</t>
+          <t>"&lt;p&gt;Dear {{insurerName}},&lt;/p&gt;&lt;p&gt;We advise a loss under policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; of {{insuredName}}.&lt;/p&gt;&lt;p&gt;Claim reference: {{claimNumber}}&lt;br/&gt;Date of loss: {{lossDate}} {{lossTime}}&lt;br/&gt;Place of loss: {{lossPlace}}&lt;br/&gt;Nature of loss: {{lossType}}&lt;br/&gt;Estimated amount: {{currency}} {{estimate}}&lt;/p&gt;&lt;p&gt;{{message}}&lt;/p&gt;&lt;p&gt;{{companyName}} Claims&lt;/p&gt;"</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>documents.accent_color</t>
+          <t>claims.settlement_maker_checker</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>"#1f4e79"</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>documents.acknowledgement_receipt_note</t>
+          <t>collections.email_subject</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>"This acknowledgement receipt is not an official receipt. The official receipt is issued once the payment is verified by Accounting."</t>
+          <t>"Premium payment reminder - Policy {{policyNumber}}"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>documents.default_logo_path</t>
+          <t>collections.email_template</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>"assets/iorta-technxt.png"</t>
+          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;This is a reminder that the premium of &lt;b&gt;{{amount}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; (bill {{billNumber}}), due on {{dueDate}}, has not yet been received.&lt;/p&gt;&lt;p&gt;Please disregard this notice if payment has been made.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>documents.default_signatory</t>
+          <t>collections.reminder_days_before</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>""</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>documents.payment_instructions</t>
+          <t>collections.reminder_repeat_days</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>"Please settle the total amount due on or before the due date. Make cheques payable to {{companyName}} and quote the bill number as the payment reference. For bank transfers or e-wallet payments, send the proof of payment to your account officer."</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>documents.receipt_footer</t>
+          <t>direct_bill.email_body</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>""</t>
+          <t>"&lt;p&gt;Dear {{insurerName}},&lt;/p&gt;&lt;p&gt;Please find our commission debit note &lt;b&gt;{{dnNumber}}&lt;/b&gt; for {{amount}}, due on {{dueDate}}.&lt;/p&gt;&lt;p&gt;Kindly settle the amount net of the expanded withholding tax on the commission and send BIR Form 2307 for the tax withheld.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>email.template.broker_slip_request</t>
+          <t>direct_bill.email_subject</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;We invite your quotation for the risk below.&lt;/p&gt;&lt;p&gt;Broker slip &lt;b&gt;{{slipNumber}}&lt;/b&gt;&lt;br/&gt;Insured: {{insuredName}}&lt;br/&gt;Class: {{productType}}&lt;br/&gt;Sum insured: {{currency}} {{sumInsured}}&lt;br/&gt;Period: {{period}}&lt;br/&gt;Requested covers: {{covers}}&lt;/p&gt;&lt;p&gt;Please send your terms (premium, rate, deductibles, conditions, the line you can write and the validity of the offer) by &lt;b&gt;{{responseDueDate}}&lt;/b&gt;.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Request for quotation {{slipNumber}} - {{productType}} - {{insuredName}}"}</t>
+          <t>"Commission debit note {{dnNumber}} - {{companyName}}"</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>email.template.endorsement_customer</t>
+          <t>documents.accent_color</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;We have prepared {{action}} &lt;b&gt;{{endorsementNumber}}&lt;/b&gt; on policy {{policyNumber}}. Premium adjustment: {{currency}} {{premiumDelta}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "{{companyName}}: {{action}} {{endorsementNumber}} on policy {{policyNumber}}"}</t>
+          <t>"#1f4e79"</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>email.template.insurer_submission</t>
+          <t>documents.acknowledgement_receipt_note</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;Please review quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; for {{customerName}} ({{productType}}), sum insured {{currency}} {{sumInsured}}, indicated gross premium {{currency}} {{grossPremium}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Placement request {{quotationNumber}} - {{productType}}"}</t>
+          <t>"This acknowledgement receipt is not an official receipt. The official receipt is issued once the payment is verified by Accounting."</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>email.template.placement_order</t>
+          <t>documents.default_logo_path</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;On behalf of our client we place the risk below with you and request your confirmation of cover and your policy / certificate number.&lt;/p&gt;&lt;p&gt;Placement slip &lt;b&gt;{{placementNumber}}&lt;/b&gt;&lt;br/&gt;Insured: {{insuredName}}&lt;br/&gt;Class: {{productType}}&lt;br/&gt;Period: {{period}}&lt;br/&gt;Sum insured (100%): {{currency}} {{sumInsured}}&lt;br/&gt;Your share: &lt;b&gt;{{sharePercent}}%&lt;/b&gt; ({{role}})&lt;br/&gt;Your share of sum insured: {{currency}} {{shareSumInsured}}&lt;br/&gt;Your share of premium: {{currency}} {{sharePremium}} (gross {{currency}} {{sharePremiumTotal}})&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Placement slip {{placementNumber}} - firm order - {{insuredName}}"}</t>
+          <t>"assets/iorta-technxt.png"</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>email.template.policy_issued</t>
+          <t>documents.default_signatory</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;Policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; ({{productType}}) was issued from quotation {{quotationNumber}}. Gross premium: {{currency}} {{grossPremium}}.&lt;/p&gt;", "subject": "Your policy {{policyNumber}} has been issued"}</t>
+          <t>""</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>email.template.quote_approval</t>
+          <t>documents.payment_instructions</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;Your {{productType}} quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; is ready. Gross premium: {{currency}} {{grossPremium}}.&lt;/p&gt;&lt;p&gt;&lt;a href=\"{{approvalUrl}}\"&gt;Review and accept the quotation&lt;/a&gt; (link valid for {{validHours}} hours).&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;", "subject": "{{companyName}}: please review quotation {{quotationNumber}}"}</t>
+          <t>"Please settle the total amount due on or before the due date. Make cheques payable to {{companyName}} and quote the bill number as the payment reference. For bank transfers or e-wallet payments, send the proof of payment to your account officer."</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>email.template.share_quote</t>
+          <t>documents.receipt_footer</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;{{message}}&lt;/p&gt;&lt;p&gt;Quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; ({{productType}}): gross premium {{currency}} {{grossPremium}}, valid until {{validUntil}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Your {{productType}} quotation {{quotationNumber}}"}</t>
+          <t>""</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>housekeeping.email_outbox_failed_days</t>
+          <t>email.max_attachment_mb</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>housekeeping.email_outbox_sent_days</t>
+          <t>email.template.broker_slip_request</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;We invite your quotation for the risk below.&lt;/p&gt;&lt;p&gt;Broker slip &lt;b&gt;{{slipNumber}}&lt;/b&gt;&lt;br/&gt;Insured: {{insuredName}}&lt;br/&gt;Class: {{productType}}&lt;br/&gt;Sum insured: {{currency}} {{sumInsured}}&lt;br/&gt;Period: {{period}}&lt;br/&gt;Requested covers: {{covers}}&lt;/p&gt;&lt;p&gt;Please send your terms (premium, rate, deductibles, conditions, the line you can write and the validity of the offer) by &lt;b&gt;{{responseDueDate}}&lt;/b&gt;.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Request for quotation {{slipNumber}} - {{productType}} - {{insuredName}}"}</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>housekeeping.notifications_read_days</t>
+          <t>email.template.endorsement_customer</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;We have prepared {{action}} &lt;b&gt;{{endorsementNumber}}&lt;/b&gt; on policy {{policyNumber}}. Premium adjustment: {{currency}} {{premiumDelta}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "{{companyName}}: {{action}} {{endorsementNumber}} on policy {{policyNumber}}"}</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>limits.renewal_notice_days</t>
+          <t>email.template.insurer_submission</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>[60, 30, 15]</t>
+          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;Please review quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; for {{customerName}} ({{productType}}), sum insured {{currency}} {{sumInsured}}, indicated gross premium {{currency}} {{grossPremium}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Placement request {{quotationNumber}} - {{productType}}"}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>motor.pricing_template_code</t>
+          <t>email.template.placement_order</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>"MOT-003-2025"</t>
+          <t>{"html": "&lt;p&gt;Dear {{insurerName}} underwriting team,&lt;/p&gt;&lt;p&gt;On behalf of our client we place the risk below with you and request your confirmation of cover and your policy / certificate number.&lt;/p&gt;&lt;p&gt;Placement slip &lt;b&gt;{{placementNumber}}&lt;/b&gt;&lt;br/&gt;Insured: {{insuredName}}&lt;br/&gt;Class: {{productType}}&lt;br/&gt;Period: {{period}}&lt;br/&gt;Sum insured (100%): {{currency}} {{sumInsured}}&lt;br/&gt;Your share: &lt;b&gt;{{sharePercent}}%&lt;/b&gt; ({{role}})&lt;br/&gt;Your share of sum insured: {{currency}} {{shareSumInsured}}&lt;br/&gt;Your share of premium: {{currency}} {{sharePremium}} (gross {{currency}} {{sharePremiumTotal}})&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Placement slip {{placementNumber}} - firm order - {{insuredName}}"}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>notification.approval_requests</t>
+          <t>email.template.policy_issued</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;Policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; ({{productType}}) was issued from quotation {{quotationNumber}}. Gross premium: {{currency}} {{grossPremium}}.&lt;/p&gt;", "subject": "Your policy {{policyNumber}} has been issued"}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>notification.claim_status</t>
+          <t>email.template.quote_approval</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;Your {{productType}} quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; is ready. Gross premium: {{currency}} {{grossPremium}}.&lt;/p&gt;&lt;p&gt;&lt;a href=\"{{approvalUrl}}\"&gt;Review and accept the quotation&lt;/a&gt; (link valid for {{validHours}} hours).&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;", "subject": "{{companyName}}: please review quotation {{quotationNumber}}"}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>notification.email_enabled</t>
+          <t>email.template.share_quote</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>{"html": "&lt;p&gt;Dear {{customerName}},&lt;/p&gt;&lt;p&gt;{{message}}&lt;/p&gt;&lt;p&gt;Quotation &lt;b&gt;{{quotationNumber}}&lt;/b&gt; ({{productType}}): gross premium {{currency}} {{grossPremium}}, valid until {{validUntil}}.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;", "subject": "Your {{productType}} quotation {{quotationNumber}}"}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>notification.from_address</t>
+          <t>housekeeping.email_outbox_failed_days</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>"BrokerVerse &lt;connect@iortatechnxt.com&gt;"</t>
+          <t>730</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>notification.renewal_reminder</t>
+          <t>housekeeping.email_outbox_sent_days</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>numbering.product_template.prefix</t>
+          <t>housekeeping.notifications_read_days</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>"TPL"</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>numbering.remittance_notice.prefix</t>
+          <t>limits.renewal_notice_days</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>"NTF"</t>
+          <t>[60, 30, 15]</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>product.template_statuses</t>
+          <t>motor.pricing_template_code</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>["Draft", "Active", "Inactive", "Retired"]</t>
+          <t>"MOT-003-2025"</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>remittance.bill_email_body</t>
+          <t>notification.approval_requests</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Bill {{billNumber}} dated {{billDate}}: {{currency}} {{amount}}, due {{dueDate}}.&lt;/p&gt;"</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>remittance.bill_email_subject</t>
+          <t>notification.claim_status</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>"Statement of account {{billNumber}}"</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>remittance.statement_email_body</t>
+          <t>notification.email_enabled</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Your remittance statement for {{period}} is available: &lt;a href=\"{{downloadUrl}}\"&gt;{{fileName}}&lt;/a&gt;&lt;/p&gt;"</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>remittance.statement_email_subject</t>
+          <t>notification.from_address</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>"Remittance statement {{period}}"</t>
+          <t>"BrokerVerse &lt;connect@iortatechnxt.com&gt;"</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>renewals.enforce_notice_order</t>
+          <t>notification.renewal_reminder</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -4481,113 +5414,329 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>renewals.notice_stages</t>
+          <t>numbering.product_template.prefix</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>[{"code": "first", "label": "First Notice", "stage": 1}, {"code": "second", "label": "Second Notice", "stage": 2}, {"code": "final", "label": "Final Notice", "stage": 3}]</t>
+          <t>"TPL"</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>renewals.notice_subject</t>
+          <t>numbering.remittance_notice.prefix</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>"{{noticeLabel}}: renewal of policy {{policyNumber}} (expires {{expiryDate}})"</t>
+          <t>"NTF"</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>renewals.notice_template</t>
+          <t>payments.notify_roles_on_error</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Your policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; with {{insurerName}} expires on {{expiryDate}}.&lt;/p&gt;&lt;p&gt;Renewal premium: {{currency}} {{premium}}.&lt;/p&gt;&lt;p&gt;Please contact us to renew and keep your cover in force.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+          <t>["accounting"]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>reports.email_body</t>
+          <t>product.template_statuses</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Good day,&lt;/p&gt;&lt;p&gt;The scheduled report &lt;b&gt;{{reportName}}&lt;/b&gt; for {{from}} to {{to}} is ready ({{rows}} rows, {{format}}).&lt;/p&gt;&lt;p&gt;&lt;a href=\"{{downloadUrl}}\"&gt;Download {{fileName}}&lt;/a&gt;&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+          <t>["Draft", "Active", "Inactive", "Retired"]</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>reports.email_subject</t>
+          <t>quotations.approval_link_ttl_hours</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>"{{companyName}}: {{reportName}} ({{from}} to {{to}})"</t>
+          <t>168</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>security.reset_code_max_attempts</t>
+          <t>quotations.approval_notify_roles</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>["processing"]</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>security.reset_code_minutes</t>
+          <t>receipts.email_on_record</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>security.reset_email_body</t>
+          <t>receipts.email_subject</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>"&lt;p&gt;Your verification code is &lt;b&gt;{{code}}&lt;/b&gt;. It expires in {{minutes}} minutes. If you did not ask for it, ignore this e-mail.&lt;/p&gt;"</t>
+          <t>"Official receipt {{receiptNumber}} for policy {{policyNumber}}"</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t>receipts.email_template</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Thank you for your payment. Attached is official receipt &lt;b&gt;{{receiptNumber}}&lt;/b&gt; for policy &lt;b&gt;{{policyNumber}}&lt;/b&gt;.&lt;/p&gt;&lt;table cellpadding=\"4\" style=\"border-collapse:collapse\"&gt;&lt;tr&gt;&lt;td&gt;Amount received&lt;/td&gt;&lt;td&gt;&lt;b&gt;{{amount}}&lt;/b&gt;&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Date received&lt;/td&gt;&lt;td&gt;{{receiptDate}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Mode of payment&lt;/td&gt;&lt;td&gt;{{paymentMode}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Reference&lt;/td&gt;&lt;td&gt;{{referenceNo}}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Balance remaining&lt;/td&gt;&lt;td&gt;{{balance}}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;p&gt;{{note}}&lt;/p&gt;&lt;p&gt;Please keep this receipt for your records. If you have any questions about your account, please contact your account officer.&lt;/p&gt;&lt;p&gt;Thank you,&lt;br/&gt;{{companyName}}&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>receipts.print_title</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>"Official Receipts"</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>reinsurance.treaty_requires_approval</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>remittance.bill_email_body</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Bill {{billNumber}} dated {{billDate}}: {{currency}} {{amount}}, due {{dueDate}}.&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>remittance.bill_email_subject</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>"Statement of account {{billNumber}}"</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>remittance.statement_email_body</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Your remittance statement for {{period}} is available: &lt;a href=\"{{downloadUrl}}\"&gt;{{fileName}}&lt;/a&gt;&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>remittance.statement_email_subject</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>"Remittance statement {{period}}"</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>renewals.approver_roles</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>["processing"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>renewals.enforce_notice_order</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>renewals.notice_stages</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>[{"code": "first", "label": "First Notice", "stage": 1}, {"code": "second", "label": "Second Notice", "stage": 2}, {"code": "final", "label": "Final Notice", "stage": 3}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>renewals.notice_subject</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>"{{noticeLabel}}: renewal of policy {{policyNumber}} (expires {{expiryDate}})"</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>renewals.notice_template</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Dear {{clientName}},&lt;/p&gt;&lt;p&gt;Your policy &lt;b&gt;{{policyNumber}}&lt;/b&gt; with {{insurerName}} expires on {{expiryDate}}.&lt;/p&gt;&lt;p&gt;Renewal premium: {{currency}} {{premium}}.&lt;/p&gt;&lt;p&gt;Please contact us to renew and keep your cover in force.&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>reports.download_link_ttl_hours</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>reports.email_body</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Good day,&lt;/p&gt;&lt;p&gt;The scheduled report &lt;b&gt;{{reportName}}&lt;/b&gt; for {{from}} to {{to}} is ready ({{rows}} rows, {{format}}).&lt;/p&gt;&lt;p&gt;&lt;a href=\"{{downloadUrl}}\"&gt;Download {{fileName}}&lt;/a&gt;&lt;/p&gt;&lt;p&gt;{{companyName}}&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>reports.email_subject</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>"{{companyName}}: {{reportName}} ({{from}} to {{to}})"</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>security.reset_code_max_attempts</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>security.reset_code_minutes</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>security.reset_email_body</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>"&lt;p&gt;Your verification code is &lt;b&gt;{{code}}&lt;/b&gt;. It expires in {{minutes}} minutes. If you did not ask for it, ignore this e-mail.&lt;/p&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
           <t>security.reset_email_subject</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>"Your {{companyName}} password reset code"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B52"/>
+  <autoFilter ref="A1:B70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>